<commit_message>
fix typos and include coding form file and preregistration
</commit_message>
<xml_diff>
--- a/data/es_d.xlsx
+++ b/data/es_d.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cristian/Dropbox/data_replication_centre/Cristian/power_analysis_study_2/power_analysis_project/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cristian/Dropbox/data_replication_centre/Cristian/power_analysis_study_2/reproducibility_power_analyses/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49068DEA-6246-E24F-974A-49013366ADCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2298E23F-2D09-4748-8018-B2A6C45995E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="60" yWindow="500" windowWidth="28740" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -221,24 +221,12 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -253,54 +241,39 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -608,83 +581,84 @@
   <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" style="5" customWidth="1"/>
+    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" style="6" customWidth="1"/>
     <col min="3" max="3" width="17.33203125" style="7" customWidth="1"/>
-    <col min="4" max="4" width="53.5" style="3" customWidth="1"/>
+    <col min="4" max="4" width="53.5" style="5" customWidth="1"/>
     <col min="5" max="5" width="28.83203125" style="7" customWidth="1"/>
-    <col min="6" max="6" width="29.5" customWidth="1"/>
-    <col min="7" max="7" width="41.33203125" customWidth="1"/>
+    <col min="6" max="6" width="29.5" style="8" customWidth="1"/>
+    <col min="7" max="7" width="41.33203125" style="8" customWidth="1"/>
+    <col min="8" max="16384" width="8.83203125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:7" s="4" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="7">
         <v>1.84</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:7" s="16" customFormat="1" ht="80" x14ac:dyDescent="0.2">
-      <c r="A3" s="12" t="s">
+    <row r="3" spans="1:7" ht="80" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="14">
+      <c r="B3" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="7">
         <v>0.94</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="6" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="80" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="7">
@@ -693,15 +667,15 @@
       <c r="D4" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="5" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="48" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="7">
@@ -713,7 +687,7 @@
       <c r="E5" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="8" t="s">
         <v>50</v>
       </c>
     </row>
@@ -734,77 +708,77 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="16" customFormat="1" ht="160" x14ac:dyDescent="0.2">
-      <c r="A7" s="13" t="s">
+    <row r="7" spans="1:7" ht="160" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="14">
+      <c r="B7" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="7">
         <v>3.18</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="15" t="s">
+      <c r="E7" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="6" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="192" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C8" s="7">
         <v>1</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="5" t="s">
         <v>29</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="144" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="7">
         <v>1.38</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="5" t="s">
         <v>31</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="64" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C10" s="7">
         <v>0.81</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="5" t="s">
         <v>33</v>
       </c>
       <c r="E10" s="7" t="s">
@@ -812,10 +786,10 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="48" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C11" s="7">
@@ -829,16 +803,16 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="96" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C12" s="7">
         <v>1</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="9" t="s">
         <v>37</v>
       </c>
       <c r="E12" s="7" t="s">
@@ -846,16 +820,16 @@
       </c>
     </row>
     <row r="13" spans="1:7" ht="96" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C13" s="7">
         <v>1.33</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="9" t="s">
         <v>39</v>
       </c>
       <c r="E13" s="7" t="s">
@@ -863,16 +837,16 @@
       </c>
     </row>
     <row r="14" spans="1:7" ht="112" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="6" t="s">
         <v>4</v>
       </c>
       <c r="C14" s="7">
         <v>0.998</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="5" t="s">
         <v>41</v>
       </c>
       <c r="E14" s="7" t="s">

</xml_diff>